<commit_message>
feat(export): add map ratings, phase sheets and visual excel improvements
</commit_message>
<xml_diff>
--- a/klasyfikacja.xlsx
+++ b/klasyfikacja.xlsx
@@ -12,16 +12,19 @@
     <sheet sheetId="6" name="MVP" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Double Elim" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Play-In" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Mecze" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Mapy" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="Mapy (podgląd)" state="visible" r:id="rId14"/>
+    <sheet sheetId="9" name="Mecze - Swiss 1" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Mecze - Swiss 2" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Mecze - Swiss 3" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Mecze - Playoffs" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Mapy" state="visible" r:id="rId16"/>
+    <sheet sheetId="14" name="Mapy (podgląd)" state="visible" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="53">
   <si>
     <t>User ID</t>
   </si>
@@ -128,15 +131,6 @@
     <t>Typ (seria)</t>
   </si>
   <si>
-    <t>Seria</t>
-  </si>
-  <si>
-    <t>Mapy (pkt)</t>
-  </si>
-  <si>
-    <t>Trafione mapy</t>
-  </si>
-  <si>
     <t>swiss_stage1</t>
   </si>
   <si>
@@ -149,12 +143,6 @@
     <t>1:0</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>Mecz</t>
   </si>
   <si>
@@ -173,16 +161,28 @@
     <t>OFF</t>
   </si>
   <si>
+    <t>Pkt</t>
+  </si>
+  <si>
+    <t>Ocena</t>
+  </si>
+  <si>
+    <t>BO1</t>
+  </si>
+  <si>
     <t>13:10</t>
   </si>
   <si>
     <t>13:11</t>
   </si>
   <si>
+    <t>🔥 Blisko</t>
+  </si>
+  <si>
     <t>Mapy (TYP → OFF)</t>
   </si>
   <si>
-    <t>Mapa 1: 13:10 → 13:11 (+0 pkt)</t>
+    <t>BO1: 13:10 → 13:11 (+2 pkt)</t>
   </si>
 </sst>
 </file>
@@ -201,15 +201,20 @@
       <b/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -217,16 +222,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -581,72 +602,72 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2">
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
         <v>4</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="4">
         <v>4</v>
       </c>
     </row>
@@ -659,7 +680,178 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="4" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="4" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="4" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -668,88 +860,102 @@
     <col min="6" max="6" width="5" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="6" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="20" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>444</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K2" s="4" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
-        <v>444</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="2">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="L2" s="4">
+        <v>2</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>51</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -759,53 +965,53 @@
     <col min="3" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="7" max="7" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -824,22 +1030,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -859,22 +1065,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -894,22 +1100,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -931,25 +1137,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -969,16 +1175,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -998,25 +1204,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1036,16 +1242,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1058,7 +1264,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1067,102 +1273,117 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="7" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="20" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>444</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="E2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="H2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="4">
+        <v>2</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
         <v>444</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="2">
-        <v>1</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="4">
+        <v>2</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="K3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>